<commit_message>
correction binding typeCode participant f1156a9f6edff4a450a2f67050651c045aee59c9
</commit_message>
<xml_diff>
--- a/fix/slicing-type-this/ig/StructureDefinition-fr-cda-evaluation.xlsx
+++ b/fix/slicing-type-this/ig/StructureDefinition-fr-cda-evaluation.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7492" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7493" uniqueCount="596">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-08T08:06:17+00:00</t>
+    <t>2026-10-08T10:07:19+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1100,10 +1100,13 @@
     <t>Observation.participant.typeCode</t>
   </si>
   <si>
+    <t>Code issu du JDV_HL7_v3_ParticipationType_CISIS (2.16.840.1.113883.1.11.10901).</t>
+  </si>
+  <si>
     <t>RESP</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-hl7-v3-ParticipationType-cisis|20260916095457</t>
+    <t>http://hl7.org/cda/stds/core/ValueSet/CDAParticipationType|2.0.3-sd</t>
   </si>
   <si>
     <t>Participant2.typeCode</t>
@@ -2199,7 +2202,7 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="18.49609375" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="73.28515625" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="63.4375" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
@@ -13468,7 +13471,9 @@
       <c r="K111" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="L111" s="2"/>
+      <c r="L111" t="s" s="2">
+        <v>352</v>
+      </c>
       <c r="M111" s="2"/>
       <c r="N111" s="2"/>
       <c r="O111" s="2"/>
@@ -13480,7 +13485,7 @@
         <v>75</v>
       </c>
       <c r="S111" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="T111" t="s" s="2">
         <v>75</v>
@@ -13499,7 +13504,7 @@
       </c>
       <c r="Y111" s="2"/>
       <c r="Z111" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="AA111" t="s" s="2">
         <v>75</v>
@@ -13517,7 +13522,7 @@
         <v>75</v>
       </c>
       <c r="AF111" t="s" s="2">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="AG111" t="s" s="2">
         <v>76</v>
@@ -13537,10 +13542,10 @@
     </row>
     <row r="112" hidden="true">
       <c r="A112" t="s" s="2">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -13574,7 +13579,7 @@
       </c>
       <c r="Q112" s="2"/>
       <c r="R112" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="S112" t="s" s="2">
         <v>75</v>
@@ -13596,7 +13601,7 @@
       </c>
       <c r="Y112" s="2"/>
       <c r="Z112" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="AA112" t="s" s="2">
         <v>75</v>
@@ -13614,7 +13619,7 @@
         <v>75</v>
       </c>
       <c r="AF112" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="AG112" t="s" s="2">
         <v>81</v>
@@ -13634,10 +13639,10 @@
     </row>
     <row r="113" hidden="true">
       <c r="A113" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -13713,7 +13718,7 @@
         <v>75</v>
       </c>
       <c r="AF113" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="AG113" t="s" s="2">
         <v>81</v>
@@ -13733,10 +13738,10 @@
     </row>
     <row r="114">
       <c r="A114" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -13762,10 +13767,10 @@
         <v>292</v>
       </c>
       <c r="L114" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="M114" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="N114" s="2"/>
       <c r="O114" s="2"/>
@@ -13816,7 +13821,7 @@
         <v>75</v>
       </c>
       <c r="AF114" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="AG114" t="s" s="2">
         <v>81</v>
@@ -13836,10 +13841,10 @@
     </row>
     <row r="115" hidden="true">
       <c r="A115" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
@@ -13937,10 +13942,10 @@
     </row>
     <row r="116" hidden="true">
       <c r="A116" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -13963,11 +13968,11 @@
         <v>75</v>
       </c>
       <c r="K116" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="L116" s="2"/>
       <c r="M116" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="N116" s="2"/>
       <c r="O116" s="2"/>
@@ -14018,7 +14023,7 @@
         <v>75</v>
       </c>
       <c r="AF116" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="AG116" t="s" s="2">
         <v>81</v>
@@ -14038,10 +14043,10 @@
     </row>
     <row r="117" hidden="true">
       <c r="A117" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B117" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" t="s" s="2">
@@ -14068,12 +14073,12 @@
       </c>
       <c r="L117" s="2"/>
       <c r="M117" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="N117" s="2"/>
       <c r="O117" s="2"/>
       <c r="P117" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="Q117" s="2"/>
       <c r="R117" t="s" s="2">
@@ -14099,7 +14104,7 @@
       </c>
       <c r="Y117" s="2"/>
       <c r="Z117" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="AA117" t="s" s="2">
         <v>75</v>
@@ -14117,7 +14122,7 @@
         <v>75</v>
       </c>
       <c r="AF117" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="AG117" t="s" s="2">
         <v>81</v>
@@ -14137,17 +14142,17 @@
     </row>
     <row r="118">
       <c r="A118" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B118" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C118" s="2"/>
       <c r="D118" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E118" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F118" t="s" s="2">
         <v>81</v>
@@ -14165,11 +14170,11 @@
         <v>75</v>
       </c>
       <c r="K118" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="L118" s="2"/>
       <c r="M118" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="N118" s="2"/>
       <c r="O118" s="2"/>
@@ -14220,7 +14225,7 @@
         <v>75</v>
       </c>
       <c r="AF118" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="AG118" t="s" s="2">
         <v>81</v>
@@ -14240,17 +14245,17 @@
     </row>
     <row r="119" hidden="true">
       <c r="A119" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B119" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C119" s="2"/>
       <c r="D119" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E119" t="s" s="2">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F119" t="s" s="2">
         <v>81</v>
@@ -14268,11 +14273,11 @@
         <v>75</v>
       </c>
       <c r="K119" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="L119" s="2"/>
       <c r="M119" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="N119" s="2"/>
       <c r="O119" s="2"/>
@@ -14323,7 +14328,7 @@
         <v>75</v>
       </c>
       <c r="AF119" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="AG119" t="s" s="2">
         <v>81</v>
@@ -14343,17 +14348,17 @@
     </row>
     <row r="120" hidden="true">
       <c r="A120" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B120" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C120" s="2"/>
       <c r="D120" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E120" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F120" t="s" s="2">
         <v>81</v>
@@ -14371,11 +14376,11 @@
         <v>75</v>
       </c>
       <c r="K120" t="s" s="2">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="L120" s="2"/>
       <c r="M120" t="s" s="2">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="N120" s="2"/>
       <c r="O120" s="2"/>
@@ -14426,7 +14431,7 @@
         <v>75</v>
       </c>
       <c r="AF120" t="s" s="2">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="AG120" t="s" s="2">
         <v>81</v>
@@ -14446,17 +14451,17 @@
     </row>
     <row r="121">
       <c r="A121" t="s" s="2">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B121" t="s" s="2">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C121" s="2"/>
       <c r="D121" t="s" s="2">
         <v>75</v>
       </c>
       <c r="E121" t="s" s="2">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F121" t="s" s="2">
         <v>81</v>
@@ -14474,11 +14479,11 @@
         <v>75</v>
       </c>
       <c r="K121" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="L121" s="2"/>
       <c r="M121" t="s" s="2">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="N121" s="2"/>
       <c r="O121" s="2"/>
@@ -14529,7 +14534,7 @@
         <v>75</v>
       </c>
       <c r="AF121" t="s" s="2">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="AG121" t="s" s="2">
         <v>81</v>
@@ -14549,10 +14554,10 @@
     </row>
     <row r="122" hidden="true">
       <c r="A122" t="s" s="2">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B122" t="s" s="2">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" t="s" s="2">
@@ -14628,7 +14633,7 @@
         <v>75</v>
       </c>
       <c r="AF122" t="s" s="2">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="AG122" t="s" s="2">
         <v>81</v>
@@ -14648,10 +14653,10 @@
     </row>
     <row r="123">
       <c r="A123" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B123" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" t="s" s="2">
@@ -14674,13 +14679,13 @@
         <v>75</v>
       </c>
       <c r="K123" t="s" s="2">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="L123" t="s" s="2">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="M123" t="s" s="2">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="N123" s="2"/>
       <c r="O123" s="2"/>
@@ -14731,7 +14736,7 @@
         <v>75</v>
       </c>
       <c r="AF123" t="s" s="2">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="AG123" t="s" s="2">
         <v>76</v>
@@ -14751,10 +14756,10 @@
     </row>
     <row r="124" hidden="true">
       <c r="A124" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B124" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" t="s" s="2">
@@ -14777,7 +14782,7 @@
         <v>75</v>
       </c>
       <c r="K124" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="L124" s="2"/>
       <c r="M124" s="2"/>
@@ -14818,7 +14823,7 @@
         <v>75</v>
       </c>
       <c r="AB124" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AC124" s="2"/>
       <c r="AD124" t="s" s="2">
@@ -14828,7 +14833,7 @@
         <v>125</v>
       </c>
       <c r="AF124" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="AG124" t="s" s="2">
         <v>81</v>
@@ -14848,13 +14853,13 @@
     </row>
     <row r="125" hidden="true">
       <c r="A125" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B125" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C125" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D125" t="s" s="2">
         <v>75</v>
@@ -14876,7 +14881,7 @@
         <v>75</v>
       </c>
       <c r="K125" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="L125" s="2"/>
       <c r="M125" s="2"/>
@@ -14929,7 +14934,7 @@
         <v>75</v>
       </c>
       <c r="AF125" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="AG125" t="s" s="2">
         <v>81</v>
@@ -14949,10 +14954,10 @@
     </row>
     <row r="126" hidden="true">
       <c r="A126" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B126" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" t="s" s="2">
@@ -15050,10 +15055,10 @@
     </row>
     <row r="127" hidden="true">
       <c r="A127" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B127" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C127" s="2"/>
       <c r="D127" t="s" s="2">
@@ -15151,10 +15156,10 @@
     </row>
     <row r="128" hidden="true">
       <c r="A128" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B128" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C128" s="2"/>
       <c r="D128" t="s" s="2">
@@ -15252,10 +15257,10 @@
     </row>
     <row r="129" hidden="true">
       <c r="A129" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B129" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C129" s="2"/>
       <c r="D129" t="s" s="2">
@@ -15353,10 +15358,10 @@
     </row>
     <row r="130" hidden="true">
       <c r="A130" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B130" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C130" s="2"/>
       <c r="D130" t="s" s="2">
@@ -15456,10 +15461,10 @@
     </row>
     <row r="131" hidden="true">
       <c r="A131" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B131" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C131" s="2"/>
       <c r="D131" t="s" s="2">
@@ -15559,10 +15564,10 @@
     </row>
     <row r="132" hidden="true">
       <c r="A132" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B132" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C132" s="2"/>
       <c r="D132" t="s" s="2">
@@ -15662,10 +15667,10 @@
     </row>
     <row r="133" hidden="true">
       <c r="A133" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B133" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C133" s="2"/>
       <c r="D133" t="s" s="2">
@@ -15765,10 +15770,10 @@
     </row>
     <row r="134" hidden="true">
       <c r="A134" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B134" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C134" s="2"/>
       <c r="D134" t="s" s="2">
@@ -15866,10 +15871,10 @@
     </row>
     <row r="135" hidden="true">
       <c r="A135" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B135" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C135" s="2"/>
       <c r="D135" t="s" s="2">
@@ -15906,7 +15911,7 @@
         <v>75</v>
       </c>
       <c r="S135" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="T135" t="s" s="2">
         <v>75</v>
@@ -15925,7 +15930,7 @@
       </c>
       <c r="Y135" s="2"/>
       <c r="Z135" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="AA135" t="s" s="2">
         <v>75</v>
@@ -15943,7 +15948,7 @@
         <v>75</v>
       </c>
       <c r="AF135" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="AG135" t="s" s="2">
         <v>76</v>
@@ -15963,10 +15968,10 @@
     </row>
     <row r="136" hidden="true">
       <c r="A136" t="s" s="2">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B136" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C136" s="2"/>
       <c r="D136" t="s" s="2">
@@ -15993,7 +15998,7 @@
       </c>
       <c r="L136" s="2"/>
       <c r="M136" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="N136" s="2"/>
       <c r="O136" s="2"/>
@@ -16044,7 +16049,7 @@
         <v>75</v>
       </c>
       <c r="AF136" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="AG136" t="s" s="2">
         <v>81</v>
@@ -16064,10 +16069,10 @@
     </row>
     <row r="137" hidden="true">
       <c r="A137" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B137" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C137" s="2"/>
       <c r="D137" t="s" s="2">
@@ -16094,12 +16099,12 @@
       </c>
       <c r="L137" s="2"/>
       <c r="M137" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="N137" s="2"/>
       <c r="O137" s="2"/>
       <c r="P137" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="Q137" s="2"/>
       <c r="R137" t="s" s="2">
@@ -16145,7 +16150,7 @@
         <v>75</v>
       </c>
       <c r="AF137" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="AG137" t="s" s="2">
         <v>81</v>
@@ -16165,10 +16170,10 @@
     </row>
     <row r="138" hidden="true">
       <c r="A138" t="s" s="2">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B138" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C138" s="2"/>
       <c r="D138" t="s" s="2">
@@ -16244,7 +16249,7 @@
         <v>75</v>
       </c>
       <c r="AF138" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="AG138" t="s" s="2">
         <v>81</v>
@@ -16264,10 +16269,10 @@
     </row>
     <row r="139" hidden="true">
       <c r="A139" t="s" s="2">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B139" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C139" s="2"/>
       <c r="D139" t="s" s="2">
@@ -16290,7 +16295,7 @@
         <v>75</v>
       </c>
       <c r="K139" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="L139" s="2"/>
       <c r="M139" s="2"/>
@@ -16343,7 +16348,7 @@
         <v>75</v>
       </c>
       <c r="AF139" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="AG139" t="s" s="2">
         <v>81</v>
@@ -16363,10 +16368,10 @@
     </row>
     <row r="140" hidden="true">
       <c r="A140" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B140" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C140" s="2"/>
       <c r="D140" t="s" s="2">
@@ -16389,7 +16394,7 @@
         <v>75</v>
       </c>
       <c r="K140" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="L140" s="2"/>
       <c r="M140" s="2"/>
@@ -16442,7 +16447,7 @@
         <v>75</v>
       </c>
       <c r="AF140" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="AG140" t="s" s="2">
         <v>81</v>
@@ -16462,10 +16467,10 @@
     </row>
     <row r="141" hidden="true">
       <c r="A141" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B141" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C141" s="2"/>
       <c r="D141" t="s" s="2">
@@ -16488,7 +16493,7 @@
         <v>75</v>
       </c>
       <c r="K141" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="L141" s="2"/>
       <c r="M141" s="2"/>
@@ -16541,7 +16546,7 @@
         <v>75</v>
       </c>
       <c r="AF141" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="AG141" t="s" s="2">
         <v>81</v>
@@ -16561,10 +16566,10 @@
     </row>
     <row r="142" hidden="true">
       <c r="A142" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B142" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C142" s="2"/>
       <c r="D142" t="s" s="2">
@@ -16587,7 +16592,7 @@
         <v>75</v>
       </c>
       <c r="K142" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="L142" s="2"/>
       <c r="M142" s="2"/>
@@ -16640,7 +16645,7 @@
         <v>75</v>
       </c>
       <c r="AF142" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="AG142" t="s" s="2">
         <v>81</v>
@@ -16660,10 +16665,10 @@
     </row>
     <row r="143" hidden="true">
       <c r="A143" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B143" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C143" s="2"/>
       <c r="D143" t="s" s="2">
@@ -16686,7 +16691,7 @@
         <v>75</v>
       </c>
       <c r="K143" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="L143" s="2"/>
       <c r="M143" s="2"/>
@@ -16739,7 +16744,7 @@
         <v>75</v>
       </c>
       <c r="AF143" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="AG143" t="s" s="2">
         <v>81</v>
@@ -16759,10 +16764,10 @@
     </row>
     <row r="144" hidden="true">
       <c r="A144" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B144" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C144" s="2"/>
       <c r="D144" t="s" s="2">
@@ -16785,7 +16790,7 @@
         <v>75</v>
       </c>
       <c r="K144" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="L144" s="2"/>
       <c r="M144" s="2"/>
@@ -16838,7 +16843,7 @@
         <v>75</v>
       </c>
       <c r="AF144" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="AG144" t="s" s="2">
         <v>81</v>
@@ -16858,10 +16863,10 @@
     </row>
     <row r="145" hidden="true">
       <c r="A145" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B145" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C145" s="2"/>
       <c r="D145" t="s" s="2">
@@ -16884,7 +16889,7 @@
         <v>75</v>
       </c>
       <c r="K145" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="L145" s="2"/>
       <c r="M145" s="2"/>
@@ -16937,7 +16942,7 @@
         <v>75</v>
       </c>
       <c r="AF145" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="AG145" t="s" s="2">
         <v>81</v>
@@ -16957,10 +16962,10 @@
     </row>
     <row r="146" hidden="true">
       <c r="A146" t="s" s="2">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B146" t="s" s="2">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C146" s="2"/>
       <c r="D146" t="s" s="2">
@@ -16983,7 +16988,7 @@
         <v>75</v>
       </c>
       <c r="K146" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="L146" s="2"/>
       <c r="M146" s="2"/>
@@ -17036,7 +17041,7 @@
         <v>75</v>
       </c>
       <c r="AF146" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="AG146" t="s" s="2">
         <v>81</v>
@@ -17056,10 +17061,10 @@
     </row>
     <row r="147" hidden="true">
       <c r="A147" t="s" s="2">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B147" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C147" s="2"/>
       <c r="D147" t="s" s="2">
@@ -17082,7 +17087,7 @@
         <v>75</v>
       </c>
       <c r="K147" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="L147" s="2"/>
       <c r="M147" s="2"/>
@@ -17135,7 +17140,7 @@
         <v>75</v>
       </c>
       <c r="AF147" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="AG147" t="s" s="2">
         <v>81</v>
@@ -17155,10 +17160,10 @@
     </row>
     <row r="148" hidden="true">
       <c r="A148" t="s" s="2">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B148" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C148" s="2"/>
       <c r="D148" t="s" s="2">
@@ -17181,7 +17186,7 @@
         <v>75</v>
       </c>
       <c r="K148" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="L148" s="2"/>
       <c r="M148" s="2"/>
@@ -17234,7 +17239,7 @@
         <v>75</v>
       </c>
       <c r="AF148" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="AG148" t="s" s="2">
         <v>81</v>
@@ -17254,10 +17259,10 @@
     </row>
     <row r="149" hidden="true">
       <c r="A149" t="s" s="2">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B149" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C149" s="2"/>
       <c r="D149" t="s" s="2">
@@ -17280,7 +17285,7 @@
         <v>75</v>
       </c>
       <c r="K149" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="L149" s="2"/>
       <c r="M149" s="2"/>
@@ -17333,7 +17338,7 @@
         <v>75</v>
       </c>
       <c r="AF149" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="AG149" t="s" s="2">
         <v>81</v>
@@ -17353,13 +17358,13 @@
     </row>
     <row r="150" hidden="true">
       <c r="A150" t="s" s="2">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B150" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C150" t="s" s="2">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D150" t="s" s="2">
         <v>75</v>
@@ -17381,10 +17386,10 @@
         <v>75</v>
       </c>
       <c r="K150" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="L150" t="s" s="2">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="M150" s="2"/>
       <c r="N150" s="2"/>
@@ -17436,7 +17441,7 @@
         <v>75</v>
       </c>
       <c r="AF150" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="AG150" t="s" s="2">
         <v>81</v>
@@ -17456,10 +17461,10 @@
     </row>
     <row r="151" hidden="true">
       <c r="A151" t="s" s="2">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B151" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C151" s="2"/>
       <c r="D151" t="s" s="2">
@@ -17557,10 +17562,10 @@
     </row>
     <row r="152" hidden="true">
       <c r="A152" t="s" s="2">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B152" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C152" s="2"/>
       <c r="D152" t="s" s="2">
@@ -17658,10 +17663,10 @@
     </row>
     <row r="153" hidden="true">
       <c r="A153" t="s" s="2">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B153" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C153" s="2"/>
       <c r="D153" t="s" s="2">
@@ -17759,10 +17764,10 @@
     </row>
     <row r="154" hidden="true">
       <c r="A154" t="s" s="2">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B154" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C154" s="2"/>
       <c r="D154" t="s" s="2">
@@ -17860,10 +17865,10 @@
     </row>
     <row r="155" hidden="true">
       <c r="A155" t="s" s="2">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B155" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C155" s="2"/>
       <c r="D155" t="s" s="2">
@@ -17963,10 +17968,10 @@
     </row>
     <row r="156" hidden="true">
       <c r="A156" t="s" s="2">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B156" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C156" s="2"/>
       <c r="D156" t="s" s="2">
@@ -18066,10 +18071,10 @@
     </row>
     <row r="157" hidden="true">
       <c r="A157" t="s" s="2">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B157" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C157" s="2"/>
       <c r="D157" t="s" s="2">
@@ -18169,10 +18174,10 @@
     </row>
     <row r="158" hidden="true">
       <c r="A158" t="s" s="2">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="B158" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C158" s="2"/>
       <c r="D158" t="s" s="2">
@@ -18272,10 +18277,10 @@
     </row>
     <row r="159" hidden="true">
       <c r="A159" t="s" s="2">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B159" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C159" s="2"/>
       <c r="D159" t="s" s="2">
@@ -18373,10 +18378,10 @@
     </row>
     <row r="160" hidden="true">
       <c r="A160" t="s" s="2">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B160" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C160" s="2"/>
       <c r="D160" t="s" s="2">
@@ -18413,7 +18418,7 @@
         <v>75</v>
       </c>
       <c r="S160" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="T160" t="s" s="2">
         <v>75</v>
@@ -18432,7 +18437,7 @@
       </c>
       <c r="Y160" s="2"/>
       <c r="Z160" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="AA160" t="s" s="2">
         <v>75</v>
@@ -18450,7 +18455,7 @@
         <v>75</v>
       </c>
       <c r="AF160" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="AG160" t="s" s="2">
         <v>76</v>
@@ -18470,10 +18475,10 @@
     </row>
     <row r="161" hidden="true">
       <c r="A161" t="s" s="2">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B161" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C161" s="2"/>
       <c r="D161" t="s" s="2">
@@ -18500,7 +18505,7 @@
       </c>
       <c r="L161" s="2"/>
       <c r="M161" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="N161" s="2"/>
       <c r="O161" s="2"/>
@@ -18551,7 +18556,7 @@
         <v>75</v>
       </c>
       <c r="AF161" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="AG161" t="s" s="2">
         <v>81</v>
@@ -18571,10 +18576,10 @@
     </row>
     <row r="162" hidden="true">
       <c r="A162" t="s" s="2">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B162" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C162" s="2"/>
       <c r="D162" t="s" s="2">
@@ -18601,12 +18606,12 @@
       </c>
       <c r="L162" s="2"/>
       <c r="M162" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="N162" s="2"/>
       <c r="O162" s="2"/>
       <c r="P162" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="Q162" s="2"/>
       <c r="R162" t="s" s="2">
@@ -18652,7 +18657,7 @@
         <v>75</v>
       </c>
       <c r="AF162" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="AG162" t="s" s="2">
         <v>81</v>
@@ -18672,10 +18677,10 @@
     </row>
     <row r="163" hidden="true">
       <c r="A163" t="s" s="2">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B163" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C163" s="2"/>
       <c r="D163" t="s" s="2">
@@ -18751,7 +18756,7 @@
         <v>75</v>
       </c>
       <c r="AF163" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="AG163" t="s" s="2">
         <v>81</v>
@@ -18771,10 +18776,10 @@
     </row>
     <row r="164" hidden="true">
       <c r="A164" t="s" s="2">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B164" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C164" s="2"/>
       <c r="D164" t="s" s="2">
@@ -18797,7 +18802,7 @@
         <v>75</v>
       </c>
       <c r="K164" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="L164" s="2"/>
       <c r="M164" s="2"/>
@@ -18850,7 +18855,7 @@
         <v>75</v>
       </c>
       <c r="AF164" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="AG164" t="s" s="2">
         <v>81</v>
@@ -18870,10 +18875,10 @@
     </row>
     <row r="165" hidden="true">
       <c r="A165" t="s" s="2">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B165" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C165" s="2"/>
       <c r="D165" t="s" s="2">
@@ -18896,7 +18901,7 @@
         <v>75</v>
       </c>
       <c r="K165" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="L165" s="2"/>
       <c r="M165" s="2"/>
@@ -18949,7 +18954,7 @@
         <v>75</v>
       </c>
       <c r="AF165" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="AG165" t="s" s="2">
         <v>81</v>
@@ -18969,10 +18974,10 @@
     </row>
     <row r="166" hidden="true">
       <c r="A166" t="s" s="2">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B166" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C166" s="2"/>
       <c r="D166" t="s" s="2">
@@ -18995,7 +19000,7 @@
         <v>75</v>
       </c>
       <c r="K166" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="L166" s="2"/>
       <c r="M166" s="2"/>
@@ -19048,7 +19053,7 @@
         <v>75</v>
       </c>
       <c r="AF166" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="AG166" t="s" s="2">
         <v>81</v>
@@ -19068,10 +19073,10 @@
     </row>
     <row r="167" hidden="true">
       <c r="A167" t="s" s="2">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B167" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C167" s="2"/>
       <c r="D167" t="s" s="2">
@@ -19094,7 +19099,7 @@
         <v>75</v>
       </c>
       <c r="K167" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="L167" s="2"/>
       <c r="M167" s="2"/>
@@ -19147,7 +19152,7 @@
         <v>75</v>
       </c>
       <c r="AF167" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="AG167" t="s" s="2">
         <v>81</v>
@@ -19167,10 +19172,10 @@
     </row>
     <row r="168" hidden="true">
       <c r="A168" t="s" s="2">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B168" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C168" s="2"/>
       <c r="D168" t="s" s="2">
@@ -19193,7 +19198,7 @@
         <v>75</v>
       </c>
       <c r="K168" t="s" s="2">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="L168" s="2"/>
       <c r="M168" s="2"/>
@@ -19246,7 +19251,7 @@
         <v>75</v>
       </c>
       <c r="AF168" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="AG168" t="s" s="2">
         <v>81</v>
@@ -19266,10 +19271,10 @@
     </row>
     <row r="169" hidden="true">
       <c r="A169" t="s" s="2">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B169" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C169" s="2"/>
       <c r="D169" t="s" s="2">
@@ -19292,7 +19297,7 @@
         <v>75</v>
       </c>
       <c r="K169" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="L169" s="2"/>
       <c r="M169" s="2"/>
@@ -19345,7 +19350,7 @@
         <v>75</v>
       </c>
       <c r="AF169" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="AG169" t="s" s="2">
         <v>81</v>
@@ -19365,10 +19370,10 @@
     </row>
     <row r="170" hidden="true">
       <c r="A170" t="s" s="2">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B170" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C170" s="2"/>
       <c r="D170" t="s" s="2">
@@ -19391,7 +19396,7 @@
         <v>75</v>
       </c>
       <c r="K170" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="L170" s="2"/>
       <c r="M170" s="2"/>
@@ -19444,7 +19449,7 @@
         <v>75</v>
       </c>
       <c r="AF170" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="AG170" t="s" s="2">
         <v>81</v>
@@ -19464,10 +19469,10 @@
     </row>
     <row r="171" hidden="true">
       <c r="A171" t="s" s="2">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B171" t="s" s="2">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C171" s="2"/>
       <c r="D171" t="s" s="2">
@@ -19490,7 +19495,7 @@
         <v>75</v>
       </c>
       <c r="K171" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="L171" s="2"/>
       <c r="M171" s="2"/>
@@ -19543,7 +19548,7 @@
         <v>75</v>
       </c>
       <c r="AF171" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="AG171" t="s" s="2">
         <v>81</v>
@@ -19563,10 +19568,10 @@
     </row>
     <row r="172" hidden="true">
       <c r="A172" t="s" s="2">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B172" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C172" s="2"/>
       <c r="D172" t="s" s="2">
@@ -19589,7 +19594,7 @@
         <v>75</v>
       </c>
       <c r="K172" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="L172" s="2"/>
       <c r="M172" s="2"/>
@@ -19642,7 +19647,7 @@
         <v>75</v>
       </c>
       <c r="AF172" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="AG172" t="s" s="2">
         <v>81</v>
@@ -19662,10 +19667,10 @@
     </row>
     <row r="173" hidden="true">
       <c r="A173" t="s" s="2">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B173" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C173" s="2"/>
       <c r="D173" t="s" s="2">
@@ -19688,7 +19693,7 @@
         <v>75</v>
       </c>
       <c r="K173" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="L173" s="2"/>
       <c r="M173" s="2"/>
@@ -19741,7 +19746,7 @@
         <v>75</v>
       </c>
       <c r="AF173" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="AG173" t="s" s="2">
         <v>81</v>
@@ -19761,10 +19766,10 @@
     </row>
     <row r="174" hidden="true">
       <c r="A174" t="s" s="2">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B174" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C174" s="2"/>
       <c r="D174" t="s" s="2">
@@ -19787,7 +19792,7 @@
         <v>75</v>
       </c>
       <c r="K174" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="L174" s="2"/>
       <c r="M174" s="2"/>
@@ -19840,7 +19845,7 @@
         <v>75</v>
       </c>
       <c r="AF174" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="AG174" t="s" s="2">
         <v>81</v>
@@ -19860,13 +19865,13 @@
     </row>
     <row r="175" hidden="true">
       <c r="A175" t="s" s="2">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B175" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C175" t="s" s="2">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="D175" t="s" s="2">
         <v>75</v>
@@ -19888,10 +19893,10 @@
         <v>75</v>
       </c>
       <c r="K175" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="L175" t="s" s="2">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="M175" s="2"/>
       <c r="N175" s="2"/>
@@ -19943,7 +19948,7 @@
         <v>75</v>
       </c>
       <c r="AF175" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="AG175" t="s" s="2">
         <v>81</v>
@@ -19963,10 +19968,10 @@
     </row>
     <row r="176" hidden="true">
       <c r="A176" t="s" s="2">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B176" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C176" s="2"/>
       <c r="D176" t="s" s="2">
@@ -20064,10 +20069,10 @@
     </row>
     <row r="177" hidden="true">
       <c r="A177" t="s" s="2">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B177" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C177" s="2"/>
       <c r="D177" t="s" s="2">
@@ -20165,10 +20170,10 @@
     </row>
     <row r="178" hidden="true">
       <c r="A178" t="s" s="2">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B178" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C178" s="2"/>
       <c r="D178" t="s" s="2">
@@ -20266,10 +20271,10 @@
     </row>
     <row r="179" hidden="true">
       <c r="A179" t="s" s="2">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B179" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C179" s="2"/>
       <c r="D179" t="s" s="2">
@@ -20367,10 +20372,10 @@
     </row>
     <row r="180" hidden="true">
       <c r="A180" t="s" s="2">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B180" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C180" s="2"/>
       <c r="D180" t="s" s="2">
@@ -20470,10 +20475,10 @@
     </row>
     <row r="181" hidden="true">
       <c r="A181" t="s" s="2">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B181" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C181" s="2"/>
       <c r="D181" t="s" s="2">
@@ -20573,10 +20578,10 @@
     </row>
     <row r="182" hidden="true">
       <c r="A182" t="s" s="2">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B182" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C182" s="2"/>
       <c r="D182" t="s" s="2">
@@ -20676,10 +20681,10 @@
     </row>
     <row r="183" hidden="true">
       <c r="A183" t="s" s="2">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B183" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C183" s="2"/>
       <c r="D183" t="s" s="2">
@@ -20779,10 +20784,10 @@
     </row>
     <row r="184" hidden="true">
       <c r="A184" t="s" s="2">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B184" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C184" s="2"/>
       <c r="D184" t="s" s="2">
@@ -20880,10 +20885,10 @@
     </row>
     <row r="185" hidden="true">
       <c r="A185" t="s" s="2">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B185" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C185" s="2"/>
       <c r="D185" t="s" s="2">
@@ -20920,7 +20925,7 @@
         <v>75</v>
       </c>
       <c r="S185" t="s" s="2">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="T185" t="s" s="2">
         <v>75</v>
@@ -20939,7 +20944,7 @@
       </c>
       <c r="Y185" s="2"/>
       <c r="Z185" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="AA185" t="s" s="2">
         <v>75</v>
@@ -20957,7 +20962,7 @@
         <v>75</v>
       </c>
       <c r="AF185" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="AG185" t="s" s="2">
         <v>76</v>
@@ -20977,10 +20982,10 @@
     </row>
     <row r="186" hidden="true">
       <c r="A186" t="s" s="2">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B186" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C186" s="2"/>
       <c r="D186" t="s" s="2">
@@ -21007,7 +21012,7 @@
       </c>
       <c r="L186" s="2"/>
       <c r="M186" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="N186" s="2"/>
       <c r="O186" s="2"/>
@@ -21019,7 +21024,7 @@
         <v>75</v>
       </c>
       <c r="S186" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="T186" t="s" s="2">
         <v>75</v>
@@ -21058,7 +21063,7 @@
         <v>75</v>
       </c>
       <c r="AF186" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="AG186" t="s" s="2">
         <v>81</v>
@@ -21078,10 +21083,10 @@
     </row>
     <row r="187" hidden="true">
       <c r="A187" t="s" s="2">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B187" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C187" s="2"/>
       <c r="D187" t="s" s="2">
@@ -21108,12 +21113,12 @@
       </c>
       <c r="L187" s="2"/>
       <c r="M187" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="N187" s="2"/>
       <c r="O187" s="2"/>
       <c r="P187" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="Q187" s="2"/>
       <c r="R187" t="s" s="2">
@@ -21159,7 +21164,7 @@
         <v>75</v>
       </c>
       <c r="AF187" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="AG187" t="s" s="2">
         <v>81</v>
@@ -21179,10 +21184,10 @@
     </row>
     <row r="188" hidden="true">
       <c r="A188" t="s" s="2">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B188" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C188" s="2"/>
       <c r="D188" t="s" s="2">
@@ -21258,7 +21263,7 @@
         <v>75</v>
       </c>
       <c r="AF188" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="AG188" t="s" s="2">
         <v>81</v>
@@ -21278,10 +21283,10 @@
     </row>
     <row r="189" hidden="true">
       <c r="A189" t="s" s="2">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B189" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C189" s="2"/>
       <c r="D189" t="s" s="2">
@@ -21304,7 +21309,7 @@
         <v>75</v>
       </c>
       <c r="K189" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="L189" s="2"/>
       <c r="M189" s="2"/>
@@ -21357,7 +21362,7 @@
         <v>75</v>
       </c>
       <c r="AF189" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="AG189" t="s" s="2">
         <v>81</v>
@@ -21377,10 +21382,10 @@
     </row>
     <row r="190" hidden="true">
       <c r="A190" t="s" s="2">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B190" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C190" s="2"/>
       <c r="D190" t="s" s="2">
@@ -21403,7 +21408,7 @@
         <v>75</v>
       </c>
       <c r="K190" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="L190" s="2"/>
       <c r="M190" s="2"/>
@@ -21456,7 +21461,7 @@
         <v>75</v>
       </c>
       <c r="AF190" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="AG190" t="s" s="2">
         <v>81</v>
@@ -21476,10 +21481,10 @@
     </row>
     <row r="191" hidden="true">
       <c r="A191" t="s" s="2">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B191" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C191" s="2"/>
       <c r="D191" t="s" s="2">
@@ -21502,7 +21507,7 @@
         <v>75</v>
       </c>
       <c r="K191" t="s" s="2">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="L191" s="2"/>
       <c r="M191" s="2"/>
@@ -21555,7 +21560,7 @@
         <v>75</v>
       </c>
       <c r="AF191" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="AG191" t="s" s="2">
         <v>81</v>
@@ -21575,10 +21580,10 @@
     </row>
     <row r="192" hidden="true">
       <c r="A192" t="s" s="2">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B192" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C192" s="2"/>
       <c r="D192" t="s" s="2">
@@ -21601,7 +21606,7 @@
         <v>75</v>
       </c>
       <c r="K192" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="L192" s="2"/>
       <c r="M192" s="2"/>
@@ -21654,7 +21659,7 @@
         <v>75</v>
       </c>
       <c r="AF192" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="AG192" t="s" s="2">
         <v>81</v>
@@ -21674,10 +21679,10 @@
     </row>
     <row r="193" hidden="true">
       <c r="A193" t="s" s="2">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B193" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C193" s="2"/>
       <c r="D193" t="s" s="2">
@@ -21700,7 +21705,7 @@
         <v>75</v>
       </c>
       <c r="K193" t="s" s="2">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="L193" s="2"/>
       <c r="M193" s="2"/>
@@ -21753,7 +21758,7 @@
         <v>75</v>
       </c>
       <c r="AF193" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="AG193" t="s" s="2">
         <v>81</v>
@@ -21773,10 +21778,10 @@
     </row>
     <row r="194" hidden="true">
       <c r="A194" t="s" s="2">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B194" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C194" s="2"/>
       <c r="D194" t="s" s="2">
@@ -21799,7 +21804,7 @@
         <v>75</v>
       </c>
       <c r="K194" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="L194" s="2"/>
       <c r="M194" s="2"/>
@@ -21852,7 +21857,7 @@
         <v>75</v>
       </c>
       <c r="AF194" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="AG194" t="s" s="2">
         <v>81</v>
@@ -21872,10 +21877,10 @@
     </row>
     <row r="195" hidden="true">
       <c r="A195" t="s" s="2">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B195" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C195" s="2"/>
       <c r="D195" t="s" s="2">
@@ -21898,7 +21903,7 @@
         <v>75</v>
       </c>
       <c r="K195" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="L195" s="2"/>
       <c r="M195" s="2"/>
@@ -21951,7 +21956,7 @@
         <v>75</v>
       </c>
       <c r="AF195" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="AG195" t="s" s="2">
         <v>81</v>
@@ -21971,10 +21976,10 @@
     </row>
     <row r="196" hidden="true">
       <c r="A196" t="s" s="2">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B196" t="s" s="2">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C196" s="2"/>
       <c r="D196" t="s" s="2">
@@ -21997,7 +22002,7 @@
         <v>75</v>
       </c>
       <c r="K196" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="L196" s="2"/>
       <c r="M196" s="2"/>
@@ -22050,7 +22055,7 @@
         <v>75</v>
       </c>
       <c r="AF196" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="AG196" t="s" s="2">
         <v>81</v>
@@ -22070,10 +22075,10 @@
     </row>
     <row r="197" hidden="true">
       <c r="A197" t="s" s="2">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B197" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C197" s="2"/>
       <c r="D197" t="s" s="2">
@@ -22096,7 +22101,7 @@
         <v>75</v>
       </c>
       <c r="K197" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="L197" s="2"/>
       <c r="M197" s="2"/>
@@ -22149,7 +22154,7 @@
         <v>75</v>
       </c>
       <c r="AF197" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="AG197" t="s" s="2">
         <v>81</v>
@@ -22169,10 +22174,10 @@
     </row>
     <row r="198" hidden="true">
       <c r="A198" t="s" s="2">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B198" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C198" s="2"/>
       <c r="D198" t="s" s="2">
@@ -22195,7 +22200,7 @@
         <v>75</v>
       </c>
       <c r="K198" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="L198" s="2"/>
       <c r="M198" s="2"/>
@@ -22248,7 +22253,7 @@
         <v>75</v>
       </c>
       <c r="AF198" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="AG198" t="s" s="2">
         <v>81</v>
@@ -22268,10 +22273,10 @@
     </row>
     <row r="199" hidden="true">
       <c r="A199" t="s" s="2">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B199" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C199" s="2"/>
       <c r="D199" t="s" s="2">
@@ -22294,7 +22299,7 @@
         <v>75</v>
       </c>
       <c r="K199" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="L199" s="2"/>
       <c r="M199" s="2"/>
@@ -22347,7 +22352,7 @@
         <v>75</v>
       </c>
       <c r="AF199" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="AG199" t="s" s="2">
         <v>81</v>
@@ -22367,13 +22372,13 @@
     </row>
     <row r="200" hidden="true">
       <c r="A200" t="s" s="2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B200" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C200" t="s" s="2">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="D200" t="s" s="2">
         <v>75</v>
@@ -22395,10 +22400,10 @@
         <v>75</v>
       </c>
       <c r="K200" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="L200" t="s" s="2">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="M200" s="2"/>
       <c r="N200" s="2"/>
@@ -22450,7 +22455,7 @@
         <v>75</v>
       </c>
       <c r="AF200" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="AG200" t="s" s="2">
         <v>81</v>
@@ -22470,10 +22475,10 @@
     </row>
     <row r="201" hidden="true">
       <c r="A201" t="s" s="2">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B201" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C201" s="2"/>
       <c r="D201" t="s" s="2">
@@ -22571,10 +22576,10 @@
     </row>
     <row r="202" hidden="true">
       <c r="A202" t="s" s="2">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B202" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C202" s="2"/>
       <c r="D202" t="s" s="2">
@@ -22672,10 +22677,10 @@
     </row>
     <row r="203" hidden="true">
       <c r="A203" t="s" s="2">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B203" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C203" s="2"/>
       <c r="D203" t="s" s="2">
@@ -22773,10 +22778,10 @@
     </row>
     <row r="204" hidden="true">
       <c r="A204" t="s" s="2">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B204" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C204" s="2"/>
       <c r="D204" t="s" s="2">
@@ -22874,10 +22879,10 @@
     </row>
     <row r="205" hidden="true">
       <c r="A205" t="s" s="2">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B205" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C205" s="2"/>
       <c r="D205" t="s" s="2">
@@ -22977,10 +22982,10 @@
     </row>
     <row r="206" hidden="true">
       <c r="A206" t="s" s="2">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B206" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C206" s="2"/>
       <c r="D206" t="s" s="2">
@@ -23080,10 +23085,10 @@
     </row>
     <row r="207" hidden="true">
       <c r="A207" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="B207" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C207" s="2"/>
       <c r="D207" t="s" s="2">
@@ -23183,10 +23188,10 @@
     </row>
     <row r="208" hidden="true">
       <c r="A208" t="s" s="2">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B208" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C208" s="2"/>
       <c r="D208" t="s" s="2">
@@ -23286,10 +23291,10 @@
     </row>
     <row r="209" hidden="true">
       <c r="A209" t="s" s="2">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B209" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C209" s="2"/>
       <c r="D209" t="s" s="2">
@@ -23387,10 +23392,10 @@
     </row>
     <row r="210" hidden="true">
       <c r="A210" t="s" s="2">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B210" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C210" s="2"/>
       <c r="D210" t="s" s="2">
@@ -23427,7 +23432,7 @@
         <v>75</v>
       </c>
       <c r="S210" t="s" s="2">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="T210" t="s" s="2">
         <v>75</v>
@@ -23446,7 +23451,7 @@
       </c>
       <c r="Y210" s="2"/>
       <c r="Z210" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="AA210" t="s" s="2">
         <v>75</v>
@@ -23464,7 +23469,7 @@
         <v>75</v>
       </c>
       <c r="AF210" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="AG210" t="s" s="2">
         <v>76</v>
@@ -23484,10 +23489,10 @@
     </row>
     <row r="211" hidden="true">
       <c r="A211" t="s" s="2">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B211" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C211" s="2"/>
       <c r="D211" t="s" s="2">
@@ -23514,7 +23519,7 @@
       </c>
       <c r="L211" s="2"/>
       <c r="M211" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="N211" s="2"/>
       <c r="O211" s="2"/>
@@ -23565,7 +23570,7 @@
         <v>75</v>
       </c>
       <c r="AF211" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="AG211" t="s" s="2">
         <v>81</v>
@@ -23585,10 +23590,10 @@
     </row>
     <row r="212" hidden="true">
       <c r="A212" t="s" s="2">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B212" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C212" s="2"/>
       <c r="D212" t="s" s="2">
@@ -23615,12 +23620,12 @@
       </c>
       <c r="L212" s="2"/>
       <c r="M212" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="N212" s="2"/>
       <c r="O212" s="2"/>
       <c r="P212" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="Q212" s="2"/>
       <c r="R212" t="s" s="2">
@@ -23666,7 +23671,7 @@
         <v>75</v>
       </c>
       <c r="AF212" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="AG212" t="s" s="2">
         <v>81</v>
@@ -23686,10 +23691,10 @@
     </row>
     <row r="213" hidden="true">
       <c r="A213" t="s" s="2">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B213" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C213" s="2"/>
       <c r="D213" t="s" s="2">
@@ -23765,7 +23770,7 @@
         <v>75</v>
       </c>
       <c r="AF213" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="AG213" t="s" s="2">
         <v>81</v>
@@ -23785,10 +23790,10 @@
     </row>
     <row r="214" hidden="true">
       <c r="A214" t="s" s="2">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B214" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C214" s="2"/>
       <c r="D214" t="s" s="2">
@@ -23811,7 +23816,7 @@
         <v>75</v>
       </c>
       <c r="K214" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="L214" s="2"/>
       <c r="M214" s="2"/>
@@ -23864,7 +23869,7 @@
         <v>75</v>
       </c>
       <c r="AF214" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="AG214" t="s" s="2">
         <v>81</v>
@@ -23884,10 +23889,10 @@
     </row>
     <row r="215" hidden="true">
       <c r="A215" t="s" s="2">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B215" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C215" s="2"/>
       <c r="D215" t="s" s="2">
@@ -23910,7 +23915,7 @@
         <v>75</v>
       </c>
       <c r="K215" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="L215" s="2"/>
       <c r="M215" s="2"/>
@@ -23963,7 +23968,7 @@
         <v>75</v>
       </c>
       <c r="AF215" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="AG215" t="s" s="2">
         <v>81</v>
@@ -23983,10 +23988,10 @@
     </row>
     <row r="216" hidden="true">
       <c r="A216" t="s" s="2">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B216" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C216" s="2"/>
       <c r="D216" t="s" s="2">
@@ -24009,7 +24014,7 @@
         <v>75</v>
       </c>
       <c r="K216" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="L216" s="2"/>
       <c r="M216" s="2"/>
@@ -24062,7 +24067,7 @@
         <v>75</v>
       </c>
       <c r="AF216" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="AG216" t="s" s="2">
         <v>81</v>
@@ -24082,10 +24087,10 @@
     </row>
     <row r="217" hidden="true">
       <c r="A217" t="s" s="2">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B217" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C217" s="2"/>
       <c r="D217" t="s" s="2">
@@ -24108,7 +24113,7 @@
         <v>75</v>
       </c>
       <c r="K217" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="L217" s="2"/>
       <c r="M217" s="2"/>
@@ -24161,7 +24166,7 @@
         <v>75</v>
       </c>
       <c r="AF217" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="AG217" t="s" s="2">
         <v>81</v>
@@ -24181,10 +24186,10 @@
     </row>
     <row r="218" hidden="true">
       <c r="A218" t="s" s="2">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B218" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C218" s="2"/>
       <c r="D218" t="s" s="2">
@@ -24207,7 +24212,7 @@
         <v>75</v>
       </c>
       <c r="K218" t="s" s="2">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="L218" s="2"/>
       <c r="M218" s="2"/>
@@ -24260,7 +24265,7 @@
         <v>75</v>
       </c>
       <c r="AF218" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="AG218" t="s" s="2">
         <v>81</v>
@@ -24280,10 +24285,10 @@
     </row>
     <row r="219" hidden="true">
       <c r="A219" t="s" s="2">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="B219" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C219" s="2"/>
       <c r="D219" t="s" s="2">
@@ -24306,7 +24311,7 @@
         <v>75</v>
       </c>
       <c r="K219" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="L219" s="2"/>
       <c r="M219" s="2"/>
@@ -24359,7 +24364,7 @@
         <v>75</v>
       </c>
       <c r="AF219" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="AG219" t="s" s="2">
         <v>81</v>
@@ -24379,10 +24384,10 @@
     </row>
     <row r="220" hidden="true">
       <c r="A220" t="s" s="2">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B220" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C220" s="2"/>
       <c r="D220" t="s" s="2">
@@ -24405,7 +24410,7 @@
         <v>75</v>
       </c>
       <c r="K220" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="L220" s="2"/>
       <c r="M220" s="2"/>
@@ -24458,7 +24463,7 @@
         <v>75</v>
       </c>
       <c r="AF220" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="AG220" t="s" s="2">
         <v>81</v>
@@ -24478,10 +24483,10 @@
     </row>
     <row r="221" hidden="true">
       <c r="A221" t="s" s="2">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="B221" t="s" s="2">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C221" s="2"/>
       <c r="D221" t="s" s="2">
@@ -24504,7 +24509,7 @@
         <v>75</v>
       </c>
       <c r="K221" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="L221" s="2"/>
       <c r="M221" s="2"/>
@@ -24557,7 +24562,7 @@
         <v>75</v>
       </c>
       <c r="AF221" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="AG221" t="s" s="2">
         <v>81</v>
@@ -24577,10 +24582,10 @@
     </row>
     <row r="222" hidden="true">
       <c r="A222" t="s" s="2">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B222" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C222" s="2"/>
       <c r="D222" t="s" s="2">
@@ -24603,7 +24608,7 @@
         <v>75</v>
       </c>
       <c r="K222" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="L222" s="2"/>
       <c r="M222" s="2"/>
@@ -24656,7 +24661,7 @@
         <v>75</v>
       </c>
       <c r="AF222" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="AG222" t="s" s="2">
         <v>81</v>
@@ -24676,10 +24681,10 @@
     </row>
     <row r="223" hidden="true">
       <c r="A223" t="s" s="2">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B223" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C223" s="2"/>
       <c r="D223" t="s" s="2">
@@ -24702,7 +24707,7 @@
         <v>75</v>
       </c>
       <c r="K223" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="L223" s="2"/>
       <c r="M223" s="2"/>
@@ -24755,7 +24760,7 @@
         <v>75</v>
       </c>
       <c r="AF223" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="AG223" t="s" s="2">
         <v>81</v>
@@ -24775,10 +24780,10 @@
     </row>
     <row r="224" hidden="true">
       <c r="A224" t="s" s="2">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B224" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C224" s="2"/>
       <c r="D224" t="s" s="2">
@@ -24801,7 +24806,7 @@
         <v>75</v>
       </c>
       <c r="K224" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="L224" s="2"/>
       <c r="M224" s="2"/>
@@ -24854,7 +24859,7 @@
         <v>75</v>
       </c>
       <c r="AF224" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="AG224" t="s" s="2">
         <v>81</v>
@@ -24874,10 +24879,10 @@
     </row>
     <row r="225" hidden="true">
       <c r="A225" t="s" s="2">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="B225" t="s" s="2">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C225" s="2"/>
       <c r="D225" t="s" s="2">
@@ -24900,7 +24905,7 @@
         <v>75</v>
       </c>
       <c r="K225" t="s" s="2">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="L225" s="2"/>
       <c r="M225" s="2"/>
@@ -24953,7 +24958,7 @@
         <v>75</v>
       </c>
       <c r="AF225" t="s" s="2">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="AG225" t="s" s="2">
         <v>81</v>
@@ -24973,10 +24978,10 @@
     </row>
     <row r="226" hidden="true">
       <c r="A226" t="s" s="2">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B226" t="s" s="2">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C226" s="2"/>
       <c r="D226" t="s" s="2">
@@ -24999,7 +25004,7 @@
         <v>75</v>
       </c>
       <c r="K226" t="s" s="2">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="L226" s="2"/>
       <c r="M226" s="2"/>
@@ -25052,7 +25057,7 @@
         <v>75</v>
       </c>
       <c r="AF226" t="s" s="2">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="AG226" t="s" s="2">
         <v>81</v>
@@ -25072,10 +25077,10 @@
     </row>
     <row r="227" hidden="true">
       <c r="A227" t="s" s="2">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B227" t="s" s="2">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="C227" s="2"/>
       <c r="D227" t="s" s="2">
@@ -25098,7 +25103,7 @@
         <v>75</v>
       </c>
       <c r="K227" t="s" s="2">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="L227" s="2"/>
       <c r="M227" s="2"/>
@@ -25151,7 +25156,7 @@
         <v>75</v>
       </c>
       <c r="AF227" t="s" s="2">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="AG227" t="s" s="2">
         <v>81</v>
@@ -25171,10 +25176,10 @@
     </row>
     <row r="228" hidden="true">
       <c r="A228" t="s" s="2">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B228" t="s" s="2">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C228" s="2"/>
       <c r="D228" t="s" s="2">
@@ -25197,11 +25202,11 @@
         <v>75</v>
       </c>
       <c r="K228" t="s" s="2">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="L228" s="2"/>
       <c r="M228" t="s" s="2">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="N228" s="2"/>
       <c r="O228" s="2"/>
@@ -25252,7 +25257,7 @@
         <v>75</v>
       </c>
       <c r="AF228" t="s" s="2">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="AG228" t="s" s="2">
         <v>81</v>
@@ -25272,10 +25277,10 @@
     </row>
     <row r="229" hidden="true">
       <c r="A229" t="s" s="2">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B229" t="s" s="2">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="C229" s="2"/>
       <c r="D229" t="s" s="2">
@@ -25373,10 +25378,10 @@
     </row>
     <row r="230" hidden="true">
       <c r="A230" t="s" s="2">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="B230" t="s" s="2">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C230" s="2"/>
       <c r="D230" t="s" s="2">
@@ -25474,10 +25479,10 @@
     </row>
     <row r="231" hidden="true">
       <c r="A231" t="s" s="2">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B231" t="s" s="2">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="C231" s="2"/>
       <c r="D231" t="s" s="2">
@@ -25575,10 +25580,10 @@
     </row>
     <row r="232" hidden="true">
       <c r="A232" t="s" s="2">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="B232" t="s" s="2">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="C232" s="2"/>
       <c r="D232" t="s" s="2">
@@ -25676,10 +25681,10 @@
     </row>
     <row r="233" hidden="true">
       <c r="A233" t="s" s="2">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="B233" t="s" s="2">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="C233" s="2"/>
       <c r="D233" t="s" s="2">
@@ -25779,10 +25784,10 @@
     </row>
     <row r="234" hidden="true">
       <c r="A234" t="s" s="2">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="B234" t="s" s="2">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="C234" s="2"/>
       <c r="D234" t="s" s="2">
@@ -25882,10 +25887,10 @@
     </row>
     <row r="235" hidden="true">
       <c r="A235" t="s" s="2">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="B235" t="s" s="2">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="C235" s="2"/>
       <c r="D235" t="s" s="2">
@@ -25985,10 +25990,10 @@
     </row>
     <row r="236" hidden="true">
       <c r="A236" t="s" s="2">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="B236" t="s" s="2">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="C236" s="2"/>
       <c r="D236" t="s" s="2">
@@ -26088,10 +26093,10 @@
     </row>
     <row r="237" hidden="true">
       <c r="A237" t="s" s="2">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B237" t="s" s="2">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="C237" s="2"/>
       <c r="D237" t="s" s="2">
@@ -26189,10 +26194,10 @@
     </row>
     <row r="238" hidden="true">
       <c r="A238" t="s" s="2">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B238" t="s" s="2">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C238" s="2"/>
       <c r="D238" t="s" s="2">
@@ -26226,7 +26231,7 @@
       </c>
       <c r="Q238" s="2"/>
       <c r="R238" t="s" s="2">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="S238" t="s" s="2">
         <v>75</v>
@@ -26248,7 +26253,7 @@
       </c>
       <c r="Y238" s="2"/>
       <c r="Z238" t="s" s="2">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="AA238" t="s" s="2">
         <v>75</v>
@@ -26266,7 +26271,7 @@
         <v>75</v>
       </c>
       <c r="AF238" t="s" s="2">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="AG238" t="s" s="2">
         <v>81</v>
@@ -26286,10 +26291,10 @@
     </row>
     <row r="239" hidden="true">
       <c r="A239" t="s" s="2">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="B239" t="s" s="2">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C239" s="2"/>
       <c r="D239" t="s" s="2">
@@ -26312,7 +26317,7 @@
         <v>75</v>
       </c>
       <c r="K239" t="s" s="2">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="L239" s="2"/>
       <c r="M239" s="2"/>
@@ -26365,7 +26370,7 @@
         <v>75</v>
       </c>
       <c r="AF239" t="s" s="2">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="AG239" t="s" s="2">
         <v>76</v>
@@ -26385,10 +26390,10 @@
     </row>
     <row r="240" hidden="true">
       <c r="A240" t="s" s="2">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B240" t="s" s="2">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="C240" s="2"/>
       <c r="D240" t="s" s="2">
@@ -26411,7 +26416,7 @@
         <v>75</v>
       </c>
       <c r="K240" t="s" s="2">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="L240" s="2"/>
       <c r="M240" s="2"/>
@@ -26464,7 +26469,7 @@
         <v>75</v>
       </c>
       <c r="AF240" t="s" s="2">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="AG240" t="s" s="2">
         <v>81</v>

</xml_diff>